<commit_message>
erro no credito.py e linhas a mais nos excels
</commit_message>
<xml_diff>
--- a/alunos.xlsx
+++ b/alunos.xlsx
@@ -8,47 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luisb\Desktop\Trabalho_P4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C96679B6-B89F-46F4-A7A2-CB7572E6BE6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD587A92-7353-44C2-B5C8-20986C93DA8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3030" yWindow="3030" windowWidth="21600" windowHeight="11385" xr2:uid="{71966DCF-013D-412B-AEDC-BE2199D3BEBA}"/>
+    <workbookView xWindow="3030" yWindow="3030" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>A — Aluno</t>
-  </si>
-  <si>
-    <t>B — Presenças</t>
-  </si>
-  <si>
-    <t>C — Total Aulas</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
   <si>
     <t>Aluno</t>
   </si>
@@ -59,10 +31,22 @@
     <t>Total Aulas</t>
   </si>
   <si>
+    <t>Percentagem</t>
+  </si>
+  <si>
+    <t>Situação</t>
+  </si>
+  <si>
     <t>João</t>
   </si>
   <si>
+    <t>Admitido</t>
+  </si>
+  <si>
     <t>Maria</t>
+  </si>
+  <si>
+    <t>Excluído</t>
   </si>
   <si>
     <t>Pedro</t>
@@ -78,7 +62,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -87,31 +71,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -141,12 +112,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -482,11 +450,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E77BC67B-1159-42D4-B403-DF62A1E6A3FC}">
-  <dimension ref="A1:C7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -496,71 +468,96 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    <row r="2" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="B2" s="1">
+        <v>18</v>
+      </c>
+      <c r="C2" s="1">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>90</v>
+      </c>
+      <c r="E2" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1">
+        <v>20</v>
+      </c>
+      <c r="D3">
+        <v>50</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="1">
+        <v>15</v>
+      </c>
+      <c r="C4" s="1">
+        <v>20</v>
+      </c>
+      <c r="D4">
+        <v>75</v>
+      </c>
+      <c r="E4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2">
-        <v>18</v>
-      </c>
-      <c r="C3" s="2">
+    </row>
+    <row r="5" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1">
         <v>20</v>
       </c>
+      <c r="D5">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="2">
-        <v>10</v>
-      </c>
-      <c r="C4" s="2">
+    <row r="6" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="1">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2">
-        <v>15</v>
-      </c>
-      <c r="C5" s="2">
+      <c r="C6" s="1">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="2">
-        <v>7</v>
-      </c>
-      <c r="C6" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="2">
-        <v>20</v>
-      </c>
-      <c r="C7" s="2">
-        <v>20</v>
+      <c r="D6">
+        <v>100</v>
+      </c>
+      <c r="E6" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Parte 2 do trabalho - melhoria do codigo anterior
</commit_message>
<xml_diff>
--- a/alunos.xlsx
+++ b/alunos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luisb\Desktop\Trabalho_P4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD587A92-7353-44C2-B5C8-20986C93DA8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C70332C0-B6ED-40F1-94E8-1475AE2EAE9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3030" yWindow="3030" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Aluno</t>
   </si>
@@ -31,22 +31,10 @@
     <t>Total Aulas</t>
   </si>
   <si>
-    <t>Percentagem</t>
-  </si>
-  <si>
-    <t>Situação</t>
-  </si>
-  <si>
     <t>João</t>
   </si>
   <si>
-    <t>Admitido</t>
-  </si>
-  <si>
     <t>Maria</t>
-  </si>
-  <si>
-    <t>Excluído</t>
   </si>
   <si>
     <t>Pedro</t>
@@ -451,14 +439,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="15.5703125" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -468,16 +456,10 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="B2" s="1">
         <v>18</v>
@@ -485,16 +467,10 @@
       <c r="C2" s="1">
         <v>20</v>
       </c>
-      <c r="D2">
-        <v>90</v>
-      </c>
-      <c r="E2" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B3" s="1">
         <v>10</v>
@@ -502,16 +478,10 @@
       <c r="C3" s="1">
         <v>20</v>
       </c>
-      <c r="D3">
-        <v>50</v>
-      </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B4" s="1">
         <v>15</v>
@@ -519,16 +489,10 @@
       <c r="C4" s="1">
         <v>20</v>
       </c>
-      <c r="D4">
-        <v>75</v>
-      </c>
-      <c r="E4" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="B5" s="1">
         <v>7</v>
@@ -536,28 +500,16 @@
       <c r="C5" s="1">
         <v>20</v>
       </c>
-      <c r="D5">
-        <v>35</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
-      </c>
     </row>
-    <row r="6" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1">
         <v>20</v>
       </c>
       <c r="C6" s="1">
         <v>20</v>
-      </c>
-      <c r="D6">
-        <v>100</v>
-      </c>
-      <c r="E6" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>